<commit_message>
sensitivity table was updated
</commit_message>
<xml_diff>
--- a/Illuminance_Response_Table.xlsx
+++ b/Illuminance_Response_Table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aksu\roombrightening\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5910ED67-5C67-49D9-921C-6F0BF3EB8181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{058D50F0-E723-4CD0-9972-29BAC6FABBE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1845" yWindow="-15870" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Illuminance Data" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
   <si>
     <t>E ( Illuminance)</t>
   </si>
@@ -42,9 +42,6 @@
     <t>Decades</t>
   </si>
   <si>
-    <t>Response (Diffuse)</t>
-  </si>
-  <si>
     <t>Response (Direct)</t>
   </si>
   <si>
@@ -54,9 +51,6 @@
     <t>40 lx</t>
   </si>
   <si>
-    <t>10´-13lx between(68-31), 5lx between(10-31)</t>
-  </si>
-  <si>
     <t>30lx</t>
   </si>
   <si>
@@ -64,6 +58,15 @@
   </si>
   <si>
     <t>3lx</t>
+  </si>
+  <si>
+    <t>Sensitivity (Diffuse)</t>
+  </si>
+  <si>
+    <t>4lx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13lx </t>
   </si>
 </sst>
 </file>
@@ -259,62 +262,74 @@
   </cellStyleXfs>
   <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -322,26 +337,14 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -654,255 +657,255 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="F1" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+    </row>
+    <row r="2" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="8">
+        <v>0.01</v>
+      </c>
+      <c r="B2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="C2" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="1">
+        <v>-2</v>
+      </c>
+      <c r="G2" s="2">
+        <v>-1</v>
+      </c>
+      <c r="H2" s="3">
+        <v>0</v>
+      </c>
+      <c r="I2" s="4">
         <v>1</v>
       </c>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-    </row>
-    <row r="2" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="9">
-        <v>0.01</v>
-      </c>
-      <c r="B2" s="25" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="25" t="s">
-        <v>4</v>
-      </c>
-      <c r="F2" s="2">
-        <v>-2</v>
-      </c>
-      <c r="G2" s="3">
-        <v>-1</v>
-      </c>
-      <c r="H2" s="4">
-        <v>0</v>
-      </c>
-      <c r="I2" s="5">
+      <c r="J2" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="9">
+        <v>1.47E-2</v>
+      </c>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="8">
+        <v>2.1499999999999998E-2</v>
+      </c>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="9">
+        <v>3.1600000000000003E-2</v>
+      </c>
+      <c r="B5" s="18"/>
+      <c r="C5" s="18"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="8">
+        <v>4.6399999999999997E-2</v>
+      </c>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="9">
+        <v>6.8099999999999994E-2</v>
+      </c>
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="10">
+        <f t="shared" ref="A8:A13" si="0">A2*10</f>
+        <v>0.1</v>
+      </c>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="10">
+        <f t="shared" si="0"/>
+        <v>0.14699999999999999</v>
+      </c>
+      <c r="B9" s="18"/>
+      <c r="C9" s="18"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="10">
+        <f t="shared" si="0"/>
+        <v>0.21499999999999997</v>
+      </c>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="10">
+        <f t="shared" si="0"/>
+        <v>0.31600000000000006</v>
+      </c>
+      <c r="B11" s="18"/>
+      <c r="C11" s="18"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="10">
+        <f t="shared" si="0"/>
+        <v>0.46399999999999997</v>
+      </c>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="10">
+        <f t="shared" si="0"/>
+        <v>0.68099999999999994</v>
+      </c>
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="11">
         <v>1</v>
       </c>
-      <c r="J2" s="6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="10">
-        <v>1.47E-2</v>
-      </c>
-      <c r="B3" s="27"/>
-      <c r="C3" s="27"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="9">
-        <v>2.1499999999999998E-2</v>
-      </c>
-      <c r="B4" s="27"/>
-      <c r="C4" s="27"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="10">
-        <v>3.1600000000000003E-2</v>
-      </c>
-      <c r="B5" s="27"/>
-      <c r="C5" s="27"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="9">
-        <v>4.6399999999999997E-2</v>
-      </c>
-      <c r="B6" s="27"/>
-      <c r="C6" s="27"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="10">
-        <v>6.8099999999999994E-2</v>
-      </c>
-      <c r="B7" s="27"/>
-      <c r="C7" s="27"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="11">
-        <f>A2*10</f>
-        <v>0.1</v>
-      </c>
-      <c r="B8" s="27"/>
-      <c r="C8" s="27"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="11">
-        <f>A3*10</f>
-        <v>0.14699999999999999</v>
-      </c>
-      <c r="B9" s="27"/>
-      <c r="C9" s="27"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="11">
-        <f>A4*10</f>
-        <v>0.21499999999999997</v>
-      </c>
-      <c r="B10" s="27"/>
-      <c r="C10" s="27"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="11">
-        <f>A5*10</f>
-        <v>0.31600000000000006</v>
-      </c>
-      <c r="B11" s="27"/>
-      <c r="C11" s="27"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="11">
-        <f>A6*10</f>
-        <v>0.46399999999999997</v>
-      </c>
-      <c r="B12" s="27"/>
-      <c r="C12" s="27"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="11">
-        <f>A7*10</f>
-        <v>0.68099999999999994</v>
-      </c>
-      <c r="B13" s="28"/>
-      <c r="C13" s="28"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="12">
-        <v>1</v>
-      </c>
       <c r="B14" s="26" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C14" s="26" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="13">
+      <c r="A15" s="12">
         <v>1.47</v>
       </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="12">
+      <c r="A16" s="11">
         <v>2.15</v>
       </c>
-      <c r="B16" s="18"/>
-      <c r="C16" s="18"/>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="13">
+      <c r="A17" s="12">
         <v>3.16</v>
       </c>
-      <c r="B17" s="18"/>
-      <c r="C17" s="18"/>
+      <c r="B17" s="27"/>
+      <c r="C17" s="27"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="12">
+      <c r="A18" s="11">
         <v>4.6399999999999997</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="C18" s="18"/>
+      <c r="B18" s="27"/>
+      <c r="C18" s="27"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="13">
+      <c r="A19" s="12">
         <v>6.81</v>
       </c>
-      <c r="B19" s="19"/>
-      <c r="C19" s="19"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="14">
+      <c r="A20" s="13">
         <v>10</v>
       </c>
-      <c r="B20" s="25" t="s">
-        <v>8</v>
-      </c>
-      <c r="C20" s="25" t="s">
+      <c r="B20" s="17" t="s">
         <v>6</v>
       </c>
+      <c r="C20" s="17" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="15">
+      <c r="A21" s="14">
         <v>14.7</v>
       </c>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
+      <c r="B21" s="24"/>
+      <c r="C21" s="24"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="14">
+      <c r="A22" s="13">
         <v>21.5</v>
       </c>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
+      <c r="B22" s="24"/>
+      <c r="C22" s="24"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="15">
+      <c r="A23" s="14">
         <v>31.6</v>
       </c>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="24"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="14">
+      <c r="A24" s="13">
         <v>46.4</v>
       </c>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
+      <c r="B24" s="24"/>
+      <c r="C24" s="24"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="15">
+      <c r="A25" s="14">
         <v>68.099999999999994</v>
       </c>
-      <c r="B25" s="21"/>
-      <c r="C25" s="21"/>
+      <c r="B25" s="25"/>
+      <c r="C25" s="25"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="16">
+      <c r="A26" s="15">
         <v>100</v>
       </c>
-      <c r="B26" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="C26" s="22" t="s">
+      <c r="B26" s="21" t="s">
         <v>5</v>
       </c>
+      <c r="C26" s="21" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="17">
+      <c r="A27" s="16">
         <v>147</v>
       </c>
-      <c r="B27" s="23"/>
-      <c r="C27" s="23"/>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="16">
+      <c r="A28" s="15">
         <v>215</v>
       </c>
-      <c r="B28" s="23"/>
-      <c r="C28" s="23"/>
+      <c r="B28" s="22"/>
+      <c r="C28" s="22"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="17">
+      <c r="A29" s="16">
         <v>316</v>
       </c>
-      <c r="B29" s="24"/>
-      <c r="C29" s="24"/>
+      <c r="B29" s="23"/>
+      <c r="C29" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>

<commit_message>
making step size adaptive too
</commit_message>
<xml_diff>
--- a/Illuminance_Response_Table.xlsx
+++ b/Illuminance_Response_Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aksu\roombrightening\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{058D50F0-E723-4CD0-9972-29BAC6FABBE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AB8D897-6075-4C66-850D-6CA7E2D71C14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="690" yWindow="600" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Illuminance Data" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
   <si>
     <t>E ( Illuminance)</t>
   </si>
@@ -45,9 +45,6 @@
     <t>Response (Direct)</t>
   </si>
   <si>
-    <t>The difference was perceived almost even for one step</t>
-  </si>
-  <si>
     <t>40 lx</t>
   </si>
   <si>
@@ -67,6 +64,12 @@
   </si>
   <si>
     <t xml:space="preserve">13lx </t>
+  </si>
+  <si>
+    <t>1lx</t>
+  </si>
+  <si>
+    <t>The difference was perceived almost every two step</t>
   </si>
 </sst>
 </file>
@@ -260,7 +263,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -344,6 +347,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -661,7 +673,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>2</v>
@@ -679,10 +691,10 @@
         <v>0.01</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="F2" s="1">
         <v>-2</v>
@@ -788,32 +800,36 @@
         <v>1</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="12">
         <v>1.47</v>
       </c>
-      <c r="B15" s="27"/>
-      <c r="C15" s="27"/>
+      <c r="B15" s="30"/>
+      <c r="C15" s="30"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="11">
         <v>2.15</v>
       </c>
-      <c r="B16" s="27"/>
-      <c r="C16" s="27"/>
+      <c r="B16" s="31"/>
+      <c r="C16" s="30"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="12">
         <v>3.16</v>
       </c>
-      <c r="B17" s="27"/>
-      <c r="C17" s="27"/>
+      <c r="B17" s="29" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="29" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
@@ -834,10 +850,10 @@
         <v>10</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -880,10 +896,10 @@
         <v>100</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -908,16 +924,18 @@
       <c r="C29" s="23"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="11">
     <mergeCell ref="B2:B13"/>
     <mergeCell ref="F1:J1"/>
     <mergeCell ref="B26:B29"/>
     <mergeCell ref="B20:B25"/>
     <mergeCell ref="C26:C29"/>
     <mergeCell ref="C20:C25"/>
-    <mergeCell ref="C14:C19"/>
-    <mergeCell ref="B14:B19"/>
     <mergeCell ref="C2:C13"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="C17:C19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
updates on sensitivitty table
</commit_message>
<xml_diff>
--- a/Illuminance_Response_Table.xlsx
+++ b/Illuminance_Response_Table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aksu\roombrightening\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AB8D897-6075-4C66-850D-6CA7E2D71C14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90D45490-A3BB-424F-9145-64AA3B1B4E77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="690" yWindow="600" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
   <si>
     <t>E ( Illuminance)</t>
   </si>
@@ -69,7 +69,10 @@
     <t>1lx</t>
   </si>
   <si>
-    <t>The difference was perceived almost every two step</t>
+    <t xml:space="preserve">The difference was perceived almost every two step. So current stimilus/2.154 </t>
+  </si>
+  <si>
+    <t>The difference was perceived almost every two step. So current stimilus/2.154</t>
   </si>
 </sst>
 </file>
@@ -340,16 +343,16 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -665,7 +668,7 @@
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="20.5703125" customWidth="1"/>
+    <col min="3" max="3" width="29.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="16.5" x14ac:dyDescent="0.25">
@@ -694,7 +697,7 @@
         <v>11</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F2" s="1">
         <v>-2</v>
@@ -799,10 +802,10 @@
       <c r="A14" s="11">
         <v>1</v>
       </c>
-      <c r="B14" s="26" t="s">
+      <c r="B14" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="26" t="s">
+      <c r="C14" s="29" t="s">
         <v>10</v>
       </c>
     </row>
@@ -824,10 +827,10 @@
       <c r="A17" s="12">
         <v>3.16</v>
       </c>
-      <c r="B17" s="29" t="s">
+      <c r="B17" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="C17" s="29" t="s">
+      <c r="C17" s="26" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>